<commit_message>
fix: it is shown that the predicted protein abundance is not stable???
</commit_message>
<xml_diff>
--- a/examples/result/abundance_before_and_after_MOMA.xlsx
+++ b/examples/result/abundance_before_and_after_MOMA.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>RPE_inferred_0</t>
+          <t>ALCD2x_inferred_2</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -456,111 +456,111 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>GND</t>
+          <t>D_LACt2_inferred_1</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001458502409816422</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001438237871778059</v>
+        <v>9.220147023538615e-14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>GLUN_inferred_0</t>
+          <t>NADTRHD_inferred_0</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1.192999614868652e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>FUM_inferred_0</t>
+          <t>ACALD_inferred_1</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0001415211359701157</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001413483697054076</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>ACKr_inferred_1</t>
+          <t>PDH_inferred_0</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>0.0005504375955339479</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.0005481058796294939</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>RPI_inferred_1</t>
+          <t>PGM_inferred_1</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.729610918373964e-05</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>2.728913693702178e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>ICDHyr</t>
+          <t>TKT2_inferred_1</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>6.078295446603822e-05</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>6.076258044635506e-05</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>GLUDy</t>
+          <t>PGK</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.002725192558800741</v>
       </c>
       <c r="C9" t="n">
-        <v>1.094962006897156e-07</v>
+        <v>0.002710366497584169</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>GLCpts_inferred_0</t>
+          <t>MALt2_2_inferred_0</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.001599695246031017</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0.001581355308447866</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>PPS_inferred_0</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -573,7 +573,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>ACONTb_inferred_1</t>
+          <t>PIt2r_inferred_0</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -586,20 +586,20 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>GAPD</t>
+          <t>PGI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.003413735767989334</v>
+        <v>0.0008702157886094624</v>
       </c>
       <c r="C13" t="n">
-        <v>0.003465385474778703</v>
+        <v>0.002610000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>TKT1_inferred_0</t>
+          <t>FRD7_inferred_0</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -612,7 +612,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>FBA_inferred_1</t>
+          <t>TKT2_inferred_0</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -625,33 +625,33 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>PFK</t>
+          <t>SUCCt2_2_inferred_0</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0001664668646619976</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0001664661389358101</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>dummy_enzyme</t>
+          <t>GLUN_inferred_0</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.05212726885793511</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>0.04970709079886804</v>
+        <v>5.471975623557004e-09</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>RPI_inferred_0</t>
+          <t>PPC</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -664,7 +664,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>MALS_inferred_1</t>
+          <t>PYK_inferred_1</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -677,98 +677,98 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>ACKr_inferred_0</t>
+          <t>rib</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>0.00180459114975865</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>0.001960977087767997</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>FBP_inferred_1</t>
+          <t>TKT1_inferred_1</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>7.847113771798822e-05</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>7.84372055689017e-05</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>ENO</t>
+          <t>rnap</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.004967956445840744</v>
+        <v>3.391862675825035e-06</v>
       </c>
       <c r="C22" t="n">
-        <v>0.00477506681258781</v>
+        <v>3.518431302366667e-06</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>PGM_inferred_2</t>
+          <t>RPE_inferred_1</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0003659701022328416</v>
+        <v>4.476708021422067e-05</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0003636114086468413</v>
+        <v>4.475968114077396e-05</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>SUCCt2_2_inferred_0</t>
+          <t>GLUt2r_inferred_0</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>9.470486184649758e-08</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>PYK_inferred_1</t>
+          <t>GLCpts_inferred_0</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>0.001598126474406089</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>0.001583119854853154</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>TALA_inferred_0</t>
+          <t>FRUpts2_inferred_0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3.83268882538662e-05</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>3.831001028749806e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>ACONTa_inferred_1</t>
+          <t>PFL_inferred_0</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -781,111 +781,111 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>GLNabc_inferred_0</t>
+          <t>AKGDH_inferred_0</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>0.0005591353959620864</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>0.0005569528595562951</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>FORti_inferred_1</t>
+          <t>ACONTa_inferred_1</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>1.16015815861758e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>MALS_inferred_0</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>0.001456416235710018</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.001438192853583527</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>GLUN_inferred_1</t>
+          <t>PGM_inferred_0</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>1.172326477473035e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>TKT1_inferred_1</t>
+          <t>GLNabc_inferred_0</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7.858355315822381e-05</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>7.854039090663659e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>ACONTb_inferred_0</t>
+          <t>CYTBD_inferred_0</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>0.002806560153495526</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>0.002818183086972169</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>PYK_inferred_0</t>
+          <t>RPE_inferred_0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.0002655513648862127</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>0.0002651161029154339</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>RPE_inferred_1</t>
+          <t>MALS_inferred_0</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4.483122173003737e-05</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>4.482085026659695e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>AKGt2r_inferred_0</t>
+          <t>ACKr_inferred_1</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -898,20 +898,20 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>GLUt2r_inferred_0</t>
+          <t>PTAr_inferred_0</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>1.047075275028997e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>ACONTa_inferred_0</t>
+          <t>ICDHyr</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -924,241 +924,241 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>ALCD2x_inferred_0</t>
+          <t>GLUN_inferred_1</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>5.377151507551256e-09</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>GLUSy_inferred_0</t>
+          <t>ACONTb_inferred_1</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>-5.21472693391161e-14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>ME2_inferred_0</t>
+          <t>SUCOAS_inferred_0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.000130957275496835</v>
+        <v>0.0001992061529325677</v>
       </c>
       <c r="C41" t="n">
-        <v>0.0001308396446707918</v>
+        <v>0.0001989858018208671</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>ADK1</t>
+          <t>dummy_enzyme</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>0.05214843568649306</v>
       </c>
       <c r="C42" t="n">
-        <v>4.079664780177001e-08</v>
+        <v>0.05156819624267174</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>G6PDH2r</t>
+          <t>PTAr_inferred_1</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.0002239952250984997</v>
+        <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>0.0002235598604788606</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>TKT2_inferred_1</t>
+          <t>FORti_inferred_0</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6.087005993522135e-05</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>6.084414384942657e-05</v>
+        <v>1.109515047428059e-13</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>PDH_inferred_0</t>
+          <t>PIt2r_inferred_1</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.0005512252151221619</v>
+        <v>0.0001309158492566274</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0005483758389653158</v>
+        <v>0.0001310519628072879</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>FBA_inferred_2</t>
+          <t>G6PDH2r</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>0.0002236748327320467</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>0.0002233702432812445</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>FUM_inferred_2</t>
+          <t>FORt2_inferred_0</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>1.109515047428059e-13</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>ALCD2x_inferred_1</t>
+          <t>FORt2_inferred_1</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>1.176533531218889e-13</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>MALt2_2_inferred_0</t>
+          <t>MDH</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>0.0009350536453994707</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>0.0009282571636310589</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>GLNS_inferred_0</t>
+          <t>PPCK_inferred_0</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>9.449985421610663e-15</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>FBP_inferred_0</t>
+          <t>PGM_inferred_2</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>0.0003656547450529591</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>0.0003637312818743388</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>NADH16_inferred_0</t>
+          <t>GLNS_inferred_1</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.01361727050094248</v>
+        <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>0.01336081030140546</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>PGI</t>
+          <t>ATPS4r</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.0008708175881358341</v>
+        <v>0.01199938458195191</v>
       </c>
       <c r="C53" t="n">
-        <v>0.004973267999999975</v>
+        <v>0.01095560296712308</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>ATPS4r</t>
+          <t>LDH_D_inferred_0</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.01201232448122251</v>
+        <v>0</v>
       </c>
       <c r="C54" t="n">
-        <v>0.0107385945298983</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>GLUN_inferred_2</t>
+          <t>FBA_inferred_1</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>7.701314214672558e-09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>AKGDH_inferred_0</t>
+          <t>ACALD_inferred_0</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.0005599343714451347</v>
+        <v>0</v>
       </c>
       <c r="C56" t="n">
-        <v>0.0005572185663905891</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>ACALD_inferred_0</t>
+          <t>ICL_inferred_0</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1171,20 +1171,20 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>PGL</t>
+          <t>TPI</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.0001229874472919845</v>
+        <v>0.0004971275611280044</v>
       </c>
       <c r="C58" t="n">
-        <v>0.0001228684323847538</v>
+        <v>0.0004940700716763239</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>ALCD2x_inferred_2</t>
+          <t>FBP_inferred_1</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1197,7 +1197,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>PTAr_inferred_1</t>
+          <t>AKGt2r_inferred_0</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1210,33 +1210,33 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>TKT2_inferred_0</t>
+          <t>D_LACt2_inferred_0</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>8.732329918357651e-14</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>CYTBD_inferred_0</t>
+          <t>TALA_inferred_0</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.002809708265541164</v>
+        <v>0</v>
       </c>
       <c r="C62" t="n">
-        <v>0.002820224603522316</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>PTAr_inferred_0</t>
+          <t>THD2_inferred_0</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1249,20 +1249,20 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>SUCOAS_inferred_0</t>
+          <t>FORti_inferred_1</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.0001994908081939139</v>
+        <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>0.0001992110672058834</v>
+        <v>1.176533531218889e-13</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>FUMt2_2_inferred_0</t>
+          <t>LDH_D_inferred_1</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1275,33 +1275,33 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>FORti_inferred_0</t>
+          <t>ACKr_inferred_2</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>1.089745265153059e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>PIt2r_inferred_1</t>
+          <t>FUM_inferred_1</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.0001311840481500226</v>
+        <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>0.0001313213592341334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>PIt2r_inferred_0</t>
+          <t>ME1_inferred_0</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1314,111 +1314,111 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>rnap</t>
+          <t>NADH16_inferred_0</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3.346550298650459e-06</v>
+        <v>0.01360247738879879</v>
       </c>
       <c r="C69" t="n">
-        <v>3.346400731090445e-06</v>
+        <v>0.01349282928094323</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>PPC</t>
+          <t>SUCDi_inferred_0</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0</v>
+        <v>0.0003312870036531673</v>
       </c>
       <c r="C70" t="n">
-        <v>0</v>
+        <v>0.0003311602697492058</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>PGM_inferred_0</t>
+          <t>PGL</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0</v>
+        <v>0.0001228115317595683</v>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>0.0001227231387562963</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>ACKr_inferred_2</t>
+          <t>GAPD</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0</v>
+        <v>0.003410672836095412</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>0.003463107232982493</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>ACALD_inferred_1</t>
+          <t>FBA_inferred_0</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0</v>
+        <v>0.0002380856435428713</v>
       </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>0.0002377009687331148</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>FUM_inferred_1</t>
+          <t>GLUN_inferred_2</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>3.532359742095596e-09</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>D_LACt2_inferred_1</t>
+          <t>GLUSy_inferred_0</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>8.617889050501723e-14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>FORt2_inferred_0</t>
+          <t>FUMt2_2_inferred_0</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>1.089745265153059e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>THD2_inferred_0</t>
+          <t>ACONTb_inferred_0</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1431,46 +1431,46 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>PFL_inferred_0</t>
+          <t>GLUDy</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>9.903607706244131e-08</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>FBA_inferred_0</t>
+          <t>TALA_inferred_1</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.000238293235834436</v>
+        <v>3.874971901280573e-05</v>
       </c>
       <c r="C79" t="n">
-        <v>0.0002378212744539329</v>
+        <v>3.873174255905116e-05</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>FORt2_inferred_1</t>
+          <t>TKT1_inferred_0</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>1.16015815861758e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>LDH_D_inferred_0</t>
+          <t>ALCD2x_inferred_1</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1483,33 +1483,33 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>PGM_inferred_1</t>
+          <t>FBP_inferred_0</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>0</v>
+        <v>3.383515971594093e-15</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>ICL_inferred_0</t>
+          <t>RPI_inferred_1</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0</v>
+        <v>2.725707788024363e-05</v>
       </c>
       <c r="C83" t="n">
-        <v>0</v>
+        <v>2.725115911469206e-05</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>FRD7_inferred_0</t>
+          <t>MALS_inferred_1</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1522,33 +1522,33 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>MDH</t>
+          <t>GLNS_inferred_0</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.0009363916109983377</v>
+        <v>0</v>
       </c>
       <c r="C85" t="n">
-        <v>0.0009280766363015198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>PPCK_inferred_0</t>
+          <t>PFK</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>0.000166321844859888</v>
       </c>
       <c r="C86" t="n">
-        <v>0</v>
+        <v>0.0001663388400031148</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>GLNS_inferred_1</t>
+          <t>FUM_inferred_2</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1561,46 +1561,46 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>TPI</t>
+          <t>FUM_inferred_0</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.0004975610179634473</v>
+        <v>0.0001413191981650092</v>
       </c>
       <c r="C88" t="n">
-        <v>0.0004943925632662946</v>
+        <v>0.0001411949373328239</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>D_LACt2_inferred_0</t>
+          <t>PYK_inferred_0</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>0</v>
+        <v>0.0002653907453349407</v>
       </c>
       <c r="C89" t="n">
-        <v>0</v>
+        <v>0.0002651088650738746</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>PGK</t>
+          <t>PPS_inferred_0</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>0.002727639899723357</v>
+        <v>0</v>
       </c>
       <c r="C90" t="n">
-        <v>0.002708932562675496</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>ME1_inferred_0</t>
+          <t>ALCD2x_inferred_0</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1613,92 +1613,92 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ACONTa_inferred_0</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>0</v>
       </c>
       <c r="C92" t="n">
-        <v>9.780089337196571e-15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>LDH_D_inferred_1</t>
+          <t>ME2_inferred_0</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0</v>
+        <v>0.0001307706058225152</v>
       </c>
       <c r="C93" t="n">
-        <v>0</v>
+        <v>0.0001306926930971971</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>FRUpts2_inferred_0</t>
+          <t>ADK1</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0</v>
+        <v>3.363128935097848e-08</v>
       </c>
       <c r="C94" t="n">
-        <v>0</v>
+        <v>9.713204131389625e-08</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>rib</t>
+          <t>FBA_inferred_2</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.00177493025151612</v>
+        <v>0</v>
       </c>
       <c r="C95" t="n">
-        <v>0.001832259081461937</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>NADTRHD_inferred_0</t>
+          <t>RPI_inferred_0</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>0</v>
       </c>
       <c r="C96" t="n">
-        <v>-5.677360452579162e-14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>SUCDi_inferred_0</t>
+          <t>ACKr_inferred_0</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.0003317603956002394</v>
+        <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>0.0003315043188540608</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>TALA_inferred_1</t>
+          <t>ENO</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0</v>
+        <v>0.004963675547688186</v>
       </c>
       <c r="C98" t="n">
-        <v>0</v>
+        <v>0.004802608078769652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: further test MOMA
Next step will test MOMA using ecModels and also verified with experimental datasets.
</commit_message>
<xml_diff>
--- a/examples/result/abundance_before_and_after_MOMA.xlsx
+++ b/examples/result/abundance_before_and_after_MOMA.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>ACKr_inferred_0</t>
+          <t>PFL_inferred_0</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -469,33 +469,33 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>PGM_inferred_2</t>
+          <t>GLUN_inferred_1</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.009639699529648814</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0.006038886528515169</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>PGL</t>
+          <t>rnap</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0001225054678884098</v>
+        <v>3.717430751749394e-06</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001347423982035318</v>
+        <v>3.716923945749827e-06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>ALCD2x_inferred_2</t>
+          <t>SUCCt2_2_inferred_0</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -508,20 +508,20 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>ACONTa_inferred_1</t>
+          <t>GAPD</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.002289798083257415</v>
       </c>
       <c r="C7" t="n">
-        <v>2.033823283028653e-05</v>
+        <v>0.003388765518874096</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>GLNabc_inferred_0</t>
+          <t>AKGt2r_inferred_0</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -534,72 +534,72 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>CYTBD_inferred_0</t>
+          <t>RPE_inferred_1</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.003929677466120961</v>
+        <v>3.966810507943148e-05</v>
       </c>
       <c r="C9" t="n">
-        <v>0.003635625713916107</v>
+        <v>3.967143581727533e-05</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>MALS_inferred_0</t>
+          <t>G6PDH2r</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>0.000215675243546868</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.0002397289821056784</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>PTAr_inferred_0</t>
+          <t>PIt2r_inferred_0</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>0.0001673869754206868</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.0001663594263112718</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>GLUN_inferred_1</t>
+          <t>TKT1_inferred_1</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>7.295659663506058e-05</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>7.29588428102363e-05</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>SUCOAS_inferred_0</t>
+          <t>PTAr_inferred_0</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0005383306756000845</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0005271699252451723</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>PTAr_inferred_1</t>
+          <t>PGM_inferred_0</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -612,98 +612,98 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>G6PDH2r</t>
+          <t>FBA_inferred_2</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0002231174031144378</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.000245404343942984</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>PDH_inferred_0</t>
+          <t>MALS_inferred_0</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.001566964841966041</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>0.002362539013938209</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>TKT2_inferred_1</t>
+          <t>FUM_inferred_1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5.33797494210461e-05</v>
+        <v>0.0003499596475706666</v>
       </c>
       <c r="C17" t="n">
-        <v>5.338101213367964e-05</v>
+        <v>0.0003454681396806367</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>MALt2_2_inferred_0</t>
+          <t>TKT1_inferred_0</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1.089496192259175e-05</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>PGI</t>
+          <t>SUCOAS_inferred_0</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0006365989592024703</v>
+        <v>0.0005281740176730893</v>
       </c>
       <c r="C19" t="n">
-        <v>0.001909796877607395</v>
+        <v>0.0005179214645694791</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>ACALD_inferred_0</t>
+          <t>GLCpts_inferred_0</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>0.001192593108372567</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>0.001613833281744415</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>TKT2_inferred_0</t>
+          <t>PTAr_inferred_1</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>1.236726821715409e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>AKGt2r_inferred_0</t>
+          <t>GLNabc_inferred_0</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -716,7 +716,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>SUCCt2_2_inferred_0</t>
+          <t>ALCD2x_inferred_0</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -729,59 +729,59 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>TALA_inferred_0</t>
+          <t>CYTBD_inferred_0</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>0.003980611351002902</v>
       </c>
       <c r="C24" t="n">
-        <v>4.811120532640325e-06</v>
+        <v>0.003516546676597009</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>PYK_inferred_1</t>
+          <t>ACONTa_inferred_1</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>9.157454644573056e-05</v>
+        <v>2.603900547582251e-05</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>TKT1_inferred_1</t>
+          <t>FUM_inferred_0</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>7.587266173991202e-05</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>7.587521280831872e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>RPE_inferred_1</t>
+          <t>PGI</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4.155176316597879e-05</v>
+        <v>0.000520908107364124</v>
       </c>
       <c r="C27" t="n">
-        <v>4.15556011456151e-05</v>
+        <v>0.001562724322092368</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>GLUt2r_inferred_0</t>
+          <t>ACKr_inferred_2</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -794,53 +794,53 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>FBA_inferred_1</t>
+          <t>FUMt2_2_inferred_0</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>6.078985384686804e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>RPE_inferred_0</t>
+          <t>ALCD2x_inferred_2</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>7.507791830312958e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>FORti_inferred_1</t>
+          <t>TKT2_inferred_1</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>5.043643983422577e-05</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>5.043751333741079e-05</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>GLUN_inferred_0</t>
+          <t>ACONTa_inferred_0</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>0.000360636393148936</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>0.0003608512996383463</v>
       </c>
     </row>
     <row r="33">
@@ -859,85 +859,85 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>NADH16_inferred_0</t>
+          <t>GLUt2r_inferred_0</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.01882435952594758</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>0.01935453808447424</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>ATPS4r</t>
+          <t>ACKr_inferred_0</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.01584688809186291</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>0.01424503441657935</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>AKGDH_inferred_0</t>
+          <t>PDH_inferred_0</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.001510996176719906</v>
+        <v>0.001535981839098183</v>
       </c>
       <c r="C36" t="n">
-        <v>0.001422639920853072</v>
+        <v>0.00163704555291716</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>ACONTb_inferred_0</t>
+          <t>GLUN_inferred_2</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.0003743811858712499</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>0.000374624396506822</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>ACONTa_inferred_0</t>
+          <t>RPI_inferred_0</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.0003743811858712499</v>
+        <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>0.000374624396506822</v>
+        <v>1.181286123397043e-06</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>PYK_inferred_0</t>
+          <t>FORti_inferred_1</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8.187467237615277e-05</v>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>8.187786835973782e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>ME2_inferred_0</t>
+          <t>D_LACt2_inferred_1</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -950,20 +950,20 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>PGM_inferred_0</t>
+          <t>ME2_inferred_0</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>3.311533214243681e-05</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>3.307511462325149e-05</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>FUMt2_2_inferred_0</t>
+          <t>MALt2_2_inferred_0</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -976,98 +976,98 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>RPI_inferred_1</t>
+          <t>FUM_inferred_2</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2.933813673257723e-05</v>
+        <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>2.935244717307668e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>RPI_inferred_0</t>
+          <t>PGL</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>0.0001184192548579645</v>
       </c>
       <c r="C44" t="n">
-        <v>1.241247285627953e-06</v>
+        <v>0.0001316262680961975</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>ALCD2x_inferred_0</t>
+          <t>NADH16_inferred_0</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0</v>
+        <v>0.01830166826149126</v>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>0.01893883168671646</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>MALS_inferred_1</t>
+          <t>ALCD2x_inferred_1</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>0.0002293141690431459</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>FUM_inferred_2</t>
+          <t>AKGDH_inferred_0</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>0.001482488287440079</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.001401887531308133</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>PFK</t>
+          <t>RPE_inferred_0</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.0001292735379019455</v>
+        <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0001638243873796021</v>
+        <v>8.278028122786021e-06</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>FBA_inferred_0</t>
+          <t>GLUDy</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.0001850519003704922</v>
+        <v>2.326582415541492e-07</v>
       </c>
       <c r="C49" t="n">
-        <v>0.0001853643642977323</v>
+        <v>2.326562564051614e-07</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>GLUSy_inferred_0</t>
+          <t>PYK_inferred_1</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1080,33 +1080,33 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>GLUN_inferred_2</t>
+          <t>TALA_inferred_0</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>5.254840182381324e-06</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>GLNS_inferred_0</t>
+          <t>ACONTb_inferred_0</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0</v>
+        <v>0.000360636393148936</v>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>0.0003608512996383463</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>D_LACt2_inferred_1</t>
+          <t>ACALD_inferred_0</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1119,228 +1119,228 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>PFL_inferred_0</t>
+          <t>PFK</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0</v>
+        <v>0.0001107941513325509</v>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>0.0001648269676287393</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>GLCpts_inferred_0</t>
+          <t>GLUSy_inferred_0</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.001341876320826857</v>
+        <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>0.001613833281744359</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>GAPD</t>
+          <t>PYK_inferred_0</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.002659717737956974</v>
+        <v>9.992218021982745e-05</v>
       </c>
       <c r="C56" t="n">
-        <v>0.00337335861337973</v>
+        <v>9.955601174666429e-05</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>FUM_inferred_0</t>
+          <t>TKT2_inferred_0</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>1.37371983522759e-05</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>PPS_inferred_0</t>
+          <t>MALS_inferred_1</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
+        <v>3.627453709969894e-05</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>GLUDy</t>
+          <t>FBA_inferred_1</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2.307202348868862e-07</v>
+        <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>2.307181848337755e-07</v>
+        <v>9.540112417348724e-05</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>TKT1_inferred_0</t>
+          <t>FBA_inferred_0</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0</v>
+        <v>0.0001585991115179025</v>
       </c>
       <c r="C60" t="n">
-        <v>9.97473028620104e-06</v>
+        <v>0.0001588176688171337</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>FBA_inferred_2</t>
+          <t>RPI_inferred_1</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0</v>
+        <v>2.870414152310724e-05</v>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>2.871690080686412e-05</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>ADK1</t>
+          <t>ATPS4r</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>3.64653170530239e-08</v>
+        <v>0.0161364159730496</v>
       </c>
       <c r="C62" t="n">
-        <v>3.631070257877289e-08</v>
+        <v>0.01406117722094628</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>PIt2r_inferred_0</t>
+          <t>PGM_inferred_2</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.0001672516962315643</v>
+        <v>0.01107796724633987</v>
       </c>
       <c r="C63" t="n">
-        <v>0.0001661743843347947</v>
+        <v>0.006568345179034391</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ADK1</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.001138899003636571</v>
+        <v>3.642670220929363e-08</v>
       </c>
       <c r="C64" t="n">
-        <v>0.001198842048841591</v>
+        <v>3.566207754328043e-08</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>FUM_inferred_1</t>
+          <t>GLNS_inferred_0</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.0002610313695014076</v>
+        <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>0.0002584072769391307</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>PGK</t>
+          <t>LDH_D_inferred_1</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.002125165132017933</v>
+        <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>0.002695377784130467</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>MDH</t>
+          <t>PPCK_inferred_0</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.003338892258091421</v>
+        <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>0.003256403812691146</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>TPI</t>
+          <t>ACALD_inferred_1</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.0003863920501225859</v>
+        <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>0.000489662787350144</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>LDH_D_inferred_0</t>
+          <t>rib</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>0.001807169000135692</v>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>0.001699022204399278</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>ICL_inferred_0</t>
+          <t>THD2_inferred_0</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>0.0001807984466502759</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>FRD7_inferred_0</t>
+          <t>PIt2r_inferred_1</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1353,33 +1353,33 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>PGM_inferred_1</t>
+          <t>PPC</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>0.001803465765058051</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>FORti_inferred_0</t>
+          <t>NADTRHD_inferred_0</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>7.467556076035551e-05</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>FORt2_inferred_0</t>
+          <t>D_LACt2_inferred_0</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1392,20 +1392,20 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>ACKr_inferred_2</t>
+          <t>TPI</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0</v>
+        <v>0.0003311581006427464</v>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>0.0004926594488801349</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>ACALD_inferred_1</t>
+          <t>FRD7_inferred_0</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1418,7 +1418,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>FORt2_inferred_1</t>
+          <t>FORt2_inferred_0</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1431,33 +1431,33 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>ALCD2x_inferred_1</t>
+          <t>GND</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0</v>
+        <v>0.001404328428485584</v>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>0.001560949783417109</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>ACKr_inferred_1</t>
+          <t>ENO</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0</v>
+        <v>0.003132861411897481</v>
       </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>0.004891732719422434</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>PIt2r_inferred_1</t>
+          <t>PPS_inferred_0</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1470,7 +1470,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>NADTRHD_inferred_0</t>
+          <t>FORti_inferred_0</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1483,85 +1483,85 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>ACONTb_inferred_1</t>
+          <t>ICL_inferred_0</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>2.033823283028653e-05</v>
+        <v>2.85999770007644e-05</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>dummy_enzyme</t>
+          <t>LDH_D_inferred_0</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.02608584570457972</v>
+        <v>0</v>
       </c>
       <c r="C83" t="n">
-        <v>0.0256243942161999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>ICDHyr</t>
+          <t>MDH</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.002861331387454415</v>
+        <v>0.004166483691469321</v>
       </c>
       <c r="C84" t="n">
-        <v>0.002544038163009903</v>
+        <v>0.003528470754475911</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>GND</t>
+          <t>dummy_enzyme</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>0.001452786638515577</v>
+        <v>0.02603097692696294</v>
       </c>
       <c r="C85" t="n">
-        <v>0.001597903825239432</v>
+        <v>0.02562439421620003</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>THD2_inferred_0</t>
+          <t>TALA_inferred_1</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>3.602659145709253e-05</v>
       </c>
       <c r="C86" t="n">
-        <v>0.000174671723794206</v>
+        <v>3.602609908887794e-05</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>rib</t>
+          <t>SUCDi_inferred_0</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.001780926929988066</v>
+        <v>0.0006869265493249976</v>
       </c>
       <c r="C87" t="n">
-        <v>0.001695608489944436</v>
+        <v>0.0006696212814892217</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>GLNS_inferred_1</t>
+          <t>FRUpts2_inferred_0</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1574,20 +1574,20 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>PPCK_inferred_0</t>
+          <t>ACONTb_inferred_1</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>0</v>
       </c>
       <c r="C89" t="n">
-        <v>0</v>
+        <v>2.603900547582251e-05</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>D_LACt2_inferred_0</t>
+          <t>PGM_inferred_1</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1600,7 +1600,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>LDH_D_inferred_1</t>
+          <t>ME1_inferred_0</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1613,92 +1613,92 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>rnap</t>
+          <t>GLUN_inferred_0</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3.716457720236521e-06</v>
+        <v>0</v>
       </c>
       <c r="C92" t="n">
-        <v>3.71589392563037e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>ME1_inferred_0</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0</v>
+        <v>0.001097086190046046</v>
       </c>
       <c r="C93" t="n">
-        <v>0</v>
+        <v>0.001173537683442963</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>FRUpts2_inferred_0</t>
+          <t>ICDHyr</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>0</v>
+        <v>0.002756282286926332</v>
       </c>
       <c r="C94" t="n">
-        <v>0</v>
+        <v>0.00251844099242474</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>SUCDi_inferred_0</t>
+          <t>GLNS_inferred_1</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>0.0005123715810148449</v>
+        <v>0</v>
       </c>
       <c r="C95" t="n">
-        <v>0.0005022543994797851</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>TALA_inferred_1</t>
+          <t>ACKr_inferred_1</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>3.746656934860893e-05</v>
+        <v>0</v>
       </c>
       <c r="C96" t="n">
-        <v>3.746623628752565e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>ENO</t>
+          <t>FORt2_inferred_1</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>0.003707695404078452</v>
+        <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>0.004859986405066923</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>PPC</t>
+          <t>PGK</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0.0004505178580406032</v>
+        <v>0.001829592282088572</v>
       </c>
       <c r="C98" t="n">
-        <v>0.0005081152955683282</v>
+        <v>0.002707688195074325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>